<commit_message>
Cover short working and improved streamer error handling. Next steps: ensuring stock was shorted before covering and maybe using market orders.
</commit_message>
<xml_diff>
--- a/screener/daily_screener_signals/2024-11-10.xlsx
+++ b/screener/daily_screener_signals/2024-11-10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/beaubranton/projects/trading/new_vwap_spike_strategy/screener/daily_screener_signals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47955156-FB36-DC4C-9D53-52C8B4C3C95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EA0EF8-73F3-FC4E-912A-098C3B9ACF75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="36660" yWindow="-11060" windowWidth="30240" windowHeight="17900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -580,7 +580,7 @@
         <v>26</v>
       </c>
       <c r="E2">
-        <v>18.5</v>
+        <v>19.32</v>
       </c>
       <c r="F2">
         <v>29.257271172453908</v>
@@ -595,7 +595,7 @@
         <v>24</v>
       </c>
       <c r="J2">
-        <v>58.334311991384673</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>19.995646818844271</v>

</xml_diff>